<commit_message>
Add Puerto Vallarta properties 10-12 and update xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/imagenes/Puerto Vallarta Jalisco/1/Formato Puerto Vallarta.xlsx
+++ b/backend/imagenes/Puerto Vallarta Jalisco/1/Formato Puerto Vallarta.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="34">
   <si>
     <t>Ciudad</t>
   </si>
@@ -98,6 +98,21 @@
   </si>
   <si>
     <t xml:space="preserve"> alberca,cine,gym,jacuzzi,salon de fiestas, AC, terraza, rooftop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerto Vallarta </t>
+  </si>
+  <si>
+    <t>Atún 113, Las Gaviotas, 49328 Puerto Vallarta, Jal.</t>
+  </si>
+  <si>
+    <t>alberca,jacuzzi,AC,jardin,terraza, patio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alberca,gym,jacuzzi,salon de fiestas, terraza, AC, </t>
+  </si>
+  <si>
+    <t>negociable</t>
   </si>
 </sst>
 </file>
@@ -646,7 +661,7 @@
         <v>26</v>
       </c>
       <c r="C9" s="1">
-        <v>80000.0</v>
+        <v>81000.0</v>
       </c>
       <c r="D9" s="1">
         <v>4.0</v>
@@ -671,6 +686,111 @@
       </c>
       <c r="K9" s="1" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="1">
+        <v>46000.0</v>
+      </c>
+      <c r="D10" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="E10" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="F10" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="G10" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="1">
+        <v>550.0</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1">
+        <v>68000.0</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="E11" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G11" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I11" s="1">
+        <v>185.0</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="1">
+        <v>53000.0</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G12" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" s="1">
+        <v>130.0</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>